<commit_message>
Upd(be): crane prepopulated data for upd models
</commit_message>
<xml_diff>
--- a/backend/data/attachments/mobile/Liebherr_LTM1100.xlsx
+++ b/backend/data/attachments/mobile/Liebherr_LTM1100.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\crane_lifting_capacity\data\mobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D8829B4-A791-4161-B1E7-E7591456DE46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0871C383-929C-4873-A86C-5D8CCA166FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{D0CD5142-251E-41F7-B82A-77810B023ACC}"/>
+    <workbookView xWindow="38280" yWindow="-6060" windowWidth="29040" windowHeight="15840" xr2:uid="{D0CD5142-251E-41F7-B82A-77810B023ACC}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="23" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="21">
   <si>
     <t>Вылет, м</t>
   </si>
@@ -88,6 +88,15 @@
   </si>
   <si>
     <t>Спецшасси автомобильного типа</t>
+  </si>
+  <si>
+    <t>19.0</t>
+  </si>
+  <si>
+    <t>45.0</t>
+  </si>
+  <si>
+    <t>52.0</t>
   </si>
 </sst>
 </file>
@@ -646,18 +655,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -685,9 +688,6 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -706,6 +706,18 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -713,9 +725,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1033,7 +1042,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EE51D42-26F6-4CF7-9317-97080AD08893}">
   <dimension ref="A1:X38"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="28.28515625" style="1" customWidth="1"/>
@@ -1053,7 +1062,7 @@
       <c r="B1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="24" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1064,7 +1073,7 @@
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="26">
+      <c r="D2" s="24">
         <v>7949.39</v>
       </c>
     </row>
@@ -1072,10 +1081,10 @@
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="24" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1086,7 +1095,7 @@
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="24">
         <v>1064.54</v>
       </c>
     </row>
@@ -1097,101 +1106,101 @@
       <c r="B5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="40">
+      <c r="G5" s="37">
         <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="42"/>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="42"/>
-      <c r="K6" s="42"/>
-      <c r="L6" s="42"/>
-      <c r="M6" s="42"/>
-      <c r="N6" s="42"/>
-      <c r="O6" s="43"/>
+      <c r="C6" s="43"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="43"/>
+      <c r="L6" s="43"/>
+      <c r="M6" s="43"/>
+      <c r="N6" s="43"/>
+      <c r="O6" s="44"/>
     </row>
     <row r="7" spans="1:24" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="20"/>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="42"/>
-      <c r="E7" s="42"/>
-      <c r="F7" s="42"/>
-      <c r="G7" s="42"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="42"/>
-      <c r="K7" s="42"/>
-      <c r="L7" s="42"/>
-      <c r="M7" s="42"/>
-      <c r="N7" s="42"/>
-      <c r="O7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="43"/>
+      <c r="L7" s="43"/>
+      <c r="M7" s="43"/>
+      <c r="N7" s="43"/>
+      <c r="O7" s="44"/>
     </row>
     <row r="8" spans="1:24" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="40">
         <v>11.5</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="40">
         <v>15.2</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="40" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="40">
+        <v>22.7</v>
+      </c>
+      <c r="H8" s="40">
+        <v>26.4</v>
+      </c>
+      <c r="I8" s="40">
+        <v>30.1</v>
+      </c>
+      <c r="J8" s="40">
+        <v>33.9</v>
+      </c>
+      <c r="K8" s="40">
+        <v>37.6</v>
+      </c>
+      <c r="L8" s="40">
+        <v>41.3</v>
+      </c>
+      <c r="M8" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="21">
-        <v>22.7</v>
-      </c>
-      <c r="H8" s="21">
-        <v>26.4</v>
-      </c>
-      <c r="I8" s="21">
-        <v>30.1</v>
-      </c>
-      <c r="J8" s="21">
-        <v>33.9</v>
-      </c>
-      <c r="K8" s="21">
-        <v>37.6</v>
-      </c>
-      <c r="L8" s="21">
-        <v>41.3</v>
-      </c>
-      <c r="M8" s="21">
-        <v>45</v>
-      </c>
-      <c r="N8" s="21">
+      <c r="N8" s="40">
         <v>48.8</v>
       </c>
-      <c r="O8" s="34">
-        <v>52</v>
+      <c r="O8" s="41" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="27">
+      <c r="B9" s="25">
         <v>3</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="22">
         <v>95</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="23">
         <v>83</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -1229,7 +1238,7 @@
       </c>
     </row>
     <row r="10" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="30">
+      <c r="B10" s="28">
         <v>3.5</v>
       </c>
       <c r="C10" s="4">
@@ -1273,7 +1282,7 @@
       </c>
     </row>
     <row r="11" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="31">
+      <c r="B11" s="29">
         <v>4</v>
       </c>
       <c r="C11" s="7">
@@ -1317,7 +1326,7 @@
       </c>
     </row>
     <row r="12" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="30">
+      <c r="B12" s="28">
         <v>4.5</v>
       </c>
       <c r="C12" s="4">
@@ -1361,7 +1370,7 @@
       </c>
     </row>
     <row r="13" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="31">
+      <c r="B13" s="29">
         <v>5</v>
       </c>
       <c r="C13" s="7">
@@ -1403,10 +1412,10 @@
       <c r="O13" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="R13" s="29"/>
+      <c r="R13" s="27"/>
     </row>
     <row r="14" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="30">
+      <c r="B14" s="28">
         <v>6</v>
       </c>
       <c r="C14" s="4">
@@ -1450,7 +1459,7 @@
       </c>
     </row>
     <row r="15" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="31">
+      <c r="B15" s="29">
         <v>7</v>
       </c>
       <c r="C15" s="7">
@@ -1494,7 +1503,7 @@
       </c>
     </row>
     <row r="16" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="30">
+      <c r="B16" s="28">
         <v>8</v>
       </c>
       <c r="C16" s="4">
@@ -1536,12 +1545,12 @@
       <c r="O16" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="V16" s="28"/>
-      <c r="W16" s="28"/>
-      <c r="X16" s="28"/>
+      <c r="V16" s="26"/>
+      <c r="W16" s="26"/>
+      <c r="X16" s="26"/>
     </row>
     <row r="17" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="31">
+      <c r="B17" s="29">
         <v>9</v>
       </c>
       <c r="C17" s="7">
@@ -1585,7 +1594,7 @@
       </c>
     </row>
     <row r="18" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="30">
+      <c r="B18" s="28">
         <v>10</v>
       </c>
       <c r="C18" s="4" t="s">
@@ -1629,7 +1638,7 @@
       </c>
     </row>
     <row r="19" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="31">
+      <c r="B19" s="29">
         <v>12</v>
       </c>
       <c r="C19" s="7" t="s">
@@ -1673,7 +1682,7 @@
       </c>
     </row>
     <row r="20" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="30">
+      <c r="B20" s="28">
         <v>14</v>
       </c>
       <c r="C20" s="4" t="s">
@@ -1717,7 +1726,7 @@
       </c>
     </row>
     <row r="21" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="31">
+      <c r="B21" s="29">
         <v>16</v>
       </c>
       <c r="C21" s="7" t="s">
@@ -1761,7 +1770,7 @@
       </c>
     </row>
     <row r="22" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="30">
+      <c r="B22" s="28">
         <v>18</v>
       </c>
       <c r="C22" s="4" t="s">
@@ -1805,7 +1814,7 @@
       </c>
     </row>
     <row r="23" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="31">
+      <c r="B23" s="29">
         <v>20</v>
       </c>
       <c r="C23" s="7" t="s">
@@ -1849,7 +1858,7 @@
       </c>
     </row>
     <row r="24" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="30">
+      <c r="B24" s="28">
         <v>22</v>
       </c>
       <c r="C24" s="4" t="s">
@@ -1893,7 +1902,7 @@
       </c>
     </row>
     <row r="25" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="31">
+      <c r="B25" s="29">
         <v>24</v>
       </c>
       <c r="C25" s="7" t="s">
@@ -1937,7 +1946,7 @@
       </c>
     </row>
     <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="30">
+      <c r="B26" s="28">
         <v>26</v>
       </c>
       <c r="C26" s="4" t="s">
@@ -1981,7 +1990,7 @@
       </c>
     </row>
     <row r="27" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="31">
+      <c r="B27" s="29">
         <v>28</v>
       </c>
       <c r="C27" s="7" t="s">
@@ -2025,7 +2034,7 @@
       </c>
     </row>
     <row r="28" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="30">
+      <c r="B28" s="28">
         <v>30</v>
       </c>
       <c r="C28" s="4" t="s">
@@ -2069,7 +2078,7 @@
       </c>
     </row>
     <row r="29" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="32">
+      <c r="B29" s="30">
         <v>32</v>
       </c>
       <c r="C29" s="12" t="s">
@@ -2113,7 +2122,7 @@
       </c>
     </row>
     <row r="30" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="33">
+      <c r="B30" s="31">
         <v>34</v>
       </c>
       <c r="C30" s="16" t="s">
@@ -2157,7 +2166,7 @@
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="31">
+      <c r="B31" s="29">
         <v>36</v>
       </c>
       <c r="C31" s="7" t="s">
@@ -2201,7 +2210,7 @@
       </c>
     </row>
     <row r="32" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="30">
+      <c r="B32" s="28">
         <v>38</v>
       </c>
       <c r="C32" s="4" t="s">
@@ -2245,7 +2254,7 @@
       </c>
     </row>
     <row r="33" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="31">
+      <c r="B33" s="29">
         <v>40</v>
       </c>
       <c r="C33" s="7" t="s">
@@ -2289,7 +2298,7 @@
       </c>
     </row>
     <row r="34" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="30">
+      <c r="B34" s="28">
         <v>42</v>
       </c>
       <c r="C34" s="4" t="s">
@@ -2333,7 +2342,7 @@
       </c>
     </row>
     <row r="35" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="31">
+      <c r="B35" s="29">
         <v>44</v>
       </c>
       <c r="C35" s="7" t="s">
@@ -2377,7 +2386,7 @@
       </c>
     </row>
     <row r="36" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="30">
+      <c r="B36" s="28">
         <v>46</v>
       </c>
       <c r="C36" s="4" t="s">
@@ -2421,51 +2430,51 @@
       </c>
     </row>
     <row r="37" spans="2:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="35">
+      <c r="B37" s="32">
         <v>48</v>
       </c>
-      <c r="C37" s="36" t="s">
-        <v>1</v>
-      </c>
-      <c r="D37" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="E37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="F37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="G37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="H37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="I37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="J37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="K37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="L37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="M37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="N37" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="O37" s="39">
+      <c r="C37" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="E37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="F37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="G37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="H37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="I37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="J37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="K37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="L37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="M37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="N37" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="O37" s="36">
         <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="38" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B38" s="26"/>
+      <c r="B38" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>